<commit_message>
Ajoute l'analyse Livraison par transporteur
Introduit Noria Standard et Velox Express dans les données Livraison et ajoute le filtrage par transporteur, sans modifier la lecture globale "Tous". Préserve l'analyse A/B et enrichit le storytelling logistique sur les périodes commerciales clés.
</commit_message>
<xml_diff>
--- a/exports_hebdomadaires/export_2025-09-01.xlsx
+++ b/exports_hebdomadaires/export_2025-09-01.xlsx
@@ -1415,7 +1415,7 @@
       </c>
       <c r="AF9" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG9" t="n">
@@ -1610,7 +1610,7 @@
       </c>
       <c r="AF11" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG11" t="n">
@@ -1805,7 +1805,7 @@
       </c>
       <c r="AF13" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG13" t="n">
@@ -1909,7 +1909,7 @@
       </c>
       <c r="AF14" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG14" t="n">
@@ -2264,7 +2264,7 @@
       </c>
       <c r="AF17" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG17" t="n">
@@ -2482,7 +2482,7 @@
       </c>
       <c r="AF19" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG19" t="n">
@@ -2677,7 +2677,7 @@
       </c>
       <c r="AF21" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Velox Express</t>
         </is>
       </c>
       <c r="AG21" t="n">
@@ -2794,7 +2794,7 @@
       </c>
       <c r="AF22" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG22" t="n">
@@ -3225,7 +3225,7 @@
       </c>
       <c r="AF26" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG26" t="n">
@@ -3329,7 +3329,7 @@
       </c>
       <c r="AF27" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG27" t="n">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="AF31" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG31" t="n">
@@ -4076,7 +4076,7 @@
       </c>
       <c r="AF34" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG34" t="n">
@@ -4403,7 +4403,7 @@
       </c>
       <c r="AF37" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG37" t="n">
@@ -4515,7 +4515,7 @@
       </c>
       <c r="AF38" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG38" t="n">
@@ -4943,7 +4943,7 @@
       </c>
       <c r="AF42" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG42" t="n">
@@ -5404,7 +5404,7 @@
       </c>
       <c r="AF46" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG46" t="n">
@@ -5811,7 +5811,7 @@
       </c>
       <c r="AF50" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG50" t="n">
@@ -6386,7 +6386,7 @@
       </c>
       <c r="AF55" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG55" t="n">
@@ -6981,7 +6981,7 @@
       </c>
       <c r="AF61" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG61" t="n">
@@ -7093,7 +7093,7 @@
       </c>
       <c r="AF62" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG62" t="n">
@@ -7627,7 +7627,7 @@
       </c>
       <c r="AF67" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG67" t="n">
@@ -7736,7 +7736,7 @@
       </c>
       <c r="AF68" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG68" t="n">
@@ -7931,7 +7931,7 @@
       </c>
       <c r="AF70" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG70" t="n">
@@ -8136,7 +8136,7 @@
       </c>
       <c r="AF72" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG72" t="n">
@@ -8245,7 +8245,7 @@
       </c>
       <c r="AF73" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Velox Express</t>
         </is>
       </c>
       <c r="AG73" t="n">
@@ -8458,7 +8458,7 @@
       </c>
       <c r="AF75" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG75" t="n">
@@ -8567,7 +8567,7 @@
       </c>
       <c r="AF76" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG76" t="n">
@@ -8790,7 +8790,7 @@
       </c>
       <c r="AF78" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG78" t="n">
@@ -9345,7 +9345,7 @@
       </c>
       <c r="AF83" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG83" t="n">
@@ -9548,7 +9548,7 @@
       </c>
       <c r="AF85" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG85" t="n">
@@ -9657,7 +9657,7 @@
       </c>
       <c r="AF86" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG86" t="n">
@@ -9979,7 +9979,7 @@
       </c>
       <c r="AF89" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG89" t="n">
@@ -10184,7 +10184,7 @@
       </c>
       <c r="AF91" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG91" t="n">
@@ -10387,7 +10387,7 @@
       </c>
       <c r="AF93" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Velox Express</t>
         </is>
       </c>
       <c r="AG93" t="n">
@@ -10719,7 +10719,7 @@
       </c>
       <c r="AF96" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG96" t="n">
@@ -10950,7 +10950,7 @@
       </c>
       <c r="AF98" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG98" t="n">
@@ -11054,7 +11054,7 @@
       </c>
       <c r="AF99" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG99" t="n">
@@ -11158,7 +11158,7 @@
       </c>
       <c r="AF100" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG100" t="n">
@@ -11262,7 +11262,7 @@
       </c>
       <c r="AF101" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Velox Express</t>
         </is>
       </c>
       <c r="AG101" t="n">
@@ -11379,7 +11379,7 @@
       </c>
       <c r="AF102" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG102" t="n">
@@ -11693,7 +11693,7 @@
       </c>
       <c r="AF105" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG105" t="n">
@@ -11994,7 +11994,7 @@
       </c>
       <c r="AF108" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG108" t="n">
@@ -12217,7 +12217,7 @@
       </c>
       <c r="AF110" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG110" t="n">
@@ -12539,7 +12539,7 @@
       </c>
       <c r="AF113" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG113" t="n">
@@ -12648,7 +12648,7 @@
       </c>
       <c r="AF114" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG114" t="n">
@@ -12752,7 +12752,7 @@
       </c>
       <c r="AF115" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG115" t="n">
@@ -12856,7 +12856,7 @@
       </c>
       <c r="AF116" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG116" t="n">
@@ -12960,7 +12960,7 @@
       </c>
       <c r="AF117" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG117" t="n">
@@ -13186,7 +13186,7 @@
       </c>
       <c r="AF119" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG119" t="n">
@@ -13407,7 +13407,7 @@
       </c>
       <c r="AF121" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG121" t="n">
@@ -14048,7 +14048,7 @@
       </c>
       <c r="AF127" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG127" t="n">
@@ -14600,7 +14600,7 @@
       </c>
       <c r="AF132" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG132" t="n">
@@ -16445,7 +16445,7 @@
       </c>
       <c r="AF149" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG149" t="n">
@@ -17169,7 +17169,7 @@
       </c>
       <c r="AF156" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Velox Express</t>
         </is>
       </c>
       <c r="AG156" t="n">
@@ -17281,7 +17281,7 @@
       </c>
       <c r="AF157" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG157" t="n">
@@ -18730,7 +18730,7 @@
       </c>
       <c r="AF171" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG171" t="n">
@@ -18961,7 +18961,7 @@
       </c>
       <c r="AF173" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG173" t="n">
@@ -19387,7 +19387,7 @@
       </c>
       <c r="AF177" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG177" t="n">
@@ -19491,7 +19491,7 @@
       </c>
       <c r="AF178" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG178" t="n">
@@ -19924,7 +19924,7 @@
       </c>
       <c r="AF182" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG182" t="n">
@@ -20028,7 +20028,7 @@
       </c>
       <c r="AF183" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Velox Express</t>
         </is>
       </c>
       <c r="AG183" t="n">
@@ -20378,7 +20378,7 @@
       </c>
       <c r="AF186" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG186" t="n">
@@ -20697,7 +20697,7 @@
       </c>
       <c r="AF189" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG189" t="n">
@@ -21239,7 +21239,7 @@
       </c>
       <c r="AF194" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG194" t="n">
@@ -21761,7 +21761,7 @@
       </c>
       <c r="AF199" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG199" t="n">
@@ -21961,7 +21961,7 @@
       </c>
       <c r="AF201" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG201" t="n">
@@ -22176,7 +22176,7 @@
       </c>
       <c r="AF203" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG203" t="n">
@@ -22734,7 +22734,7 @@
       </c>
       <c r="AF208" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG208" t="n">
@@ -22838,7 +22838,7 @@
       </c>
       <c r="AF209" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG209" t="n">
@@ -23046,7 +23046,7 @@
       </c>
       <c r="AF211" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG211" t="n">
@@ -23606,7 +23606,7 @@
       </c>
       <c r="AF216" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG216" t="n">
@@ -24415,7 +24415,7 @@
       </c>
       <c r="AF223" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Velox Express</t>
         </is>
       </c>
       <c r="AG223" t="n">
@@ -25054,7 +25054,7 @@
       </c>
       <c r="AF229" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Velox Express</t>
         </is>
       </c>
       <c r="AG229" t="n">
@@ -25376,7 +25376,7 @@
       </c>
       <c r="AF232" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG232" t="n">
@@ -27095,7 +27095,7 @@
       </c>
       <c r="AF247" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG247" t="n">
@@ -27513,7 +27513,7 @@
       </c>
       <c r="AF251" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG251" t="n">
@@ -27949,7 +27949,7 @@
       </c>
       <c r="AF255" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Velox Express</t>
         </is>
       </c>
       <c r="AG255" t="n">
@@ -28258,7 +28258,7 @@
       </c>
       <c r="AF258" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG258" t="n">
@@ -28942,7 +28942,7 @@
       </c>
       <c r="AF264" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG264" t="n">
@@ -29676,7 +29676,7 @@
       </c>
       <c r="AF271" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG271" t="n">
@@ -30190,7 +30190,7 @@
       </c>
       <c r="AF276" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG276" t="n">
@@ -30294,7 +30294,7 @@
       </c>
       <c r="AF277" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG277" t="n">
@@ -30398,7 +30398,7 @@
       </c>
       <c r="AF278" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG278" t="n">
@@ -30515,7 +30515,7 @@
       </c>
       <c r="AF279" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Velox Express</t>
         </is>
       </c>
       <c r="AG279" t="n">
@@ -30723,7 +30723,7 @@
       </c>
       <c r="AF281" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG281" t="n">
@@ -30918,7 +30918,7 @@
       </c>
       <c r="AF283" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG283" t="n">
@@ -31994,7 +31994,7 @@
       </c>
       <c r="AF293" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Velox Express</t>
         </is>
       </c>
       <c r="AG293" t="n">
@@ -33578,7 +33578,7 @@
       </c>
       <c r="AF308" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG308" t="n">
@@ -34295,7 +34295,7 @@
       </c>
       <c r="AF315" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG315" t="n">
@@ -34498,7 +34498,7 @@
       </c>
       <c r="AF317" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG317" t="n">
@@ -35076,7 +35076,7 @@
       </c>
       <c r="AF322" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG322" t="n">
@@ -35590,7 +35590,7 @@
       </c>
       <c r="AF327" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG327" t="n">
@@ -36168,7 +36168,7 @@
       </c>
       <c r="AF332" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG332" t="n">
@@ -36459,7 +36459,7 @@
       </c>
       <c r="AF335" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG335" t="n">
@@ -36654,7 +36654,7 @@
       </c>
       <c r="AF337" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG337" t="n">
@@ -37564,7 +37564,7 @@
       </c>
       <c r="AF345" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG345" t="n">
@@ -37797,7 +37797,7 @@
       </c>
       <c r="AF347" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Velox Express</t>
         </is>
       </c>
       <c r="AG347" t="n">
@@ -38025,7 +38025,7 @@
       </c>
       <c r="AF349" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG349" t="n">
@@ -38129,7 +38129,7 @@
       </c>
       <c r="AF350" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Velox Express</t>
         </is>
       </c>
       <c r="AG350" t="n">
@@ -38433,7 +38433,7 @@
       </c>
       <c r="AF353" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Velox Express</t>
         </is>
       </c>
       <c r="AG353" t="n">
@@ -38633,7 +38633,7 @@
       </c>
       <c r="AF355" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG355" t="n">
@@ -39064,7 +39064,7 @@
       </c>
       <c r="AF359" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG359" t="n">
@@ -39300,7 +39300,7 @@
       </c>
       <c r="AF361" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG361" t="n">
@@ -39409,7 +39409,7 @@
       </c>
       <c r="AF362" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG362" t="n">
@@ -40389,7 +40389,7 @@
       </c>
       <c r="AF371" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG371" t="n">
@@ -40594,7 +40594,7 @@
       </c>
       <c r="AF373" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG373" t="n">
@@ -40913,7 +40913,7 @@
       </c>
       <c r="AF376" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG376" t="n">
@@ -41456,7 +41456,7 @@
       </c>
       <c r="AF381" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG381" t="n">
@@ -41656,7 +41656,7 @@
       </c>
       <c r="AF383" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG383" t="n">
@@ -42102,7 +42102,7 @@
       </c>
       <c r="AF387" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Velox Express</t>
         </is>
       </c>
       <c r="AG387" t="n">
@@ -42297,7 +42297,7 @@
       </c>
       <c r="AF389" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG389" t="n">
@@ -42702,7 +42702,7 @@
       </c>
       <c r="AF393" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG393" t="n">
@@ -43802,7 +43802,7 @@
       </c>
       <c r="AF403" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG403" t="n">
@@ -44344,7 +44344,7 @@
       </c>
       <c r="AF408" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG408" t="n">
@@ -44671,7 +44671,7 @@
       </c>
       <c r="AF411" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Velox Express</t>
         </is>
       </c>
       <c r="AG411" t="n">
@@ -44993,7 +44993,7 @@
       </c>
       <c r="AF414" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Velox Express</t>
         </is>
       </c>
       <c r="AG414" t="n">
@@ -45341,7 +45341,7 @@
       </c>
       <c r="AF417" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG417" t="n">
@@ -45984,7 +45984,7 @@
       </c>
       <c r="AF423" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG423" t="n">
@@ -46574,7 +46574,7 @@
       </c>
       <c r="AF429" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG429" t="n">
@@ -46678,7 +46678,7 @@
       </c>
       <c r="AF430" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG430" t="n">
@@ -47664,7 +47664,7 @@
       </c>
       <c r="AF439" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG439" t="n">
@@ -47994,7 +47994,7 @@
       </c>
       <c r="AF442" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG442" t="n">
@@ -48098,7 +48098,7 @@
       </c>
       <c r="AF443" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG443" t="n">
@@ -48518,7 +48518,7 @@
       </c>
       <c r="AF447" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG447" t="n">
@@ -48964,7 +48964,7 @@
       </c>
       <c r="AF451" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG451" t="n">
@@ -49301,7 +49301,7 @@
       </c>
       <c r="AF454" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG454" t="n">
@@ -49410,7 +49410,7 @@
       </c>
       <c r="AF455" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG455" t="n">
@@ -50652,7 +50652,7 @@
       </c>
       <c r="AF466" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Velox Express</t>
         </is>
       </c>
       <c r="AG466" t="n">
@@ -50860,7 +50860,7 @@
       </c>
       <c r="AF468" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Velox Express</t>
         </is>
       </c>
       <c r="AG468" t="n">
@@ -51516,7 +51516,7 @@
       </c>
       <c r="AF474" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG474" t="n">
@@ -51830,7 +51830,7 @@
       </c>
       <c r="AF477" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG477" t="n">
@@ -52276,7 +52276,7 @@
       </c>
       <c r="AF481" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG481" t="n">
@@ -52504,7 +52504,7 @@
       </c>
       <c r="AF483" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG483" t="n">
@@ -53023,7 +53023,7 @@
       </c>
       <c r="AF488" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Velox Express</t>
         </is>
       </c>
       <c r="AG488" t="n">
@@ -53737,7 +53737,7 @@
       </c>
       <c r="AF495" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG495" t="n">
@@ -53950,7 +53950,7 @@
       </c>
       <c r="AF497" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG497" t="n">
@@ -54158,7 +54158,7 @@
       </c>
       <c r="AF499" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG499" t="n">
@@ -54506,7 +54506,7 @@
       </c>
       <c r="AF502" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG502" t="n">
@@ -54610,7 +54610,7 @@
       </c>
       <c r="AF503" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG503" t="n">
@@ -54714,7 +54714,7 @@
       </c>
       <c r="AF504" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG504" t="n">
@@ -54826,7 +54826,7 @@
       </c>
       <c r="AF505" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG505" t="n">
@@ -55039,7 +55039,7 @@
       </c>
       <c r="AF507" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG507" t="n">
@@ -55348,7 +55348,7 @@
       </c>
       <c r="AF510" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG510" t="n">
@@ -55548,7 +55548,7 @@
       </c>
       <c r="AF512" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Velox Express</t>
         </is>
       </c>
       <c r="AG512" t="n">
@@ -55652,7 +55652,7 @@
       </c>
       <c r="AF513" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG513" t="n">
@@ -56358,7 +56358,7 @@
       </c>
       <c r="AF520" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG520" t="n">
@@ -56760,7 +56760,7 @@
       </c>
       <c r="AF524" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG524" t="n">
@@ -57644,7 +57644,7 @@
       </c>
       <c r="AF532" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG532" t="n">
@@ -58222,7 +58222,7 @@
       </c>
       <c r="AF537" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG537" t="n">
@@ -58529,7 +58529,7 @@
       </c>
       <c r="AF540" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG540" t="n">
@@ -59587,7 +59587,7 @@
       </c>
       <c r="AF550" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Velox Express</t>
         </is>
       </c>
       <c r="AG550" t="n">
@@ -59810,7 +59810,7 @@
       </c>
       <c r="AF552" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG552" t="n">
@@ -59914,7 +59914,7 @@
       </c>
       <c r="AF553" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG553" t="n">
@@ -60482,7 +60482,7 @@
       </c>
       <c r="AF558" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG558" t="n">
@@ -61191,7 +61191,7 @@
       </c>
       <c r="AF565" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG565" t="n">
@@ -62439,7 +62439,7 @@
       </c>
       <c r="AF577" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG577" t="n">
@@ -62543,7 +62543,7 @@
       </c>
       <c r="AF578" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG578" t="n">
@@ -62865,7 +62865,7 @@
       </c>
       <c r="AF581" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG581" t="n">
@@ -63478,7 +63478,7 @@
       </c>
       <c r="AF587" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG587" t="n">
@@ -63987,7 +63987,7 @@
       </c>
       <c r="AF592" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG592" t="n">
@@ -64993,7 +64993,7 @@
       </c>
       <c r="AF601" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG601" t="n">
@@ -65105,7 +65105,7 @@
       </c>
       <c r="AF602" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG602" t="n">
@@ -65214,7 +65214,7 @@
       </c>
       <c r="AF603" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG603" t="n">
@@ -65969,7 +65969,7 @@
       </c>
       <c r="AF610" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Velox Express</t>
         </is>
       </c>
       <c r="AG610" t="n">
@@ -66369,7 +66369,7 @@
       </c>
       <c r="AF614" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Velox Express</t>
         </is>
       </c>
       <c r="AG614" t="n">
@@ -67161,7 +67161,7 @@
       </c>
       <c r="AF622" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG622" t="n">
@@ -67392,7 +67392,7 @@
       </c>
       <c r="AF624" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG624" t="n">
@@ -67595,7 +67595,7 @@
       </c>
       <c r="AF626" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG626" t="n">
@@ -67790,7 +67790,7 @@
       </c>
       <c r="AF628" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG628" t="n">
@@ -67899,7 +67899,7 @@
       </c>
       <c r="AF629" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG629" t="n">
@@ -68345,7 +68345,7 @@
       </c>
       <c r="AF633" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Velox Express</t>
         </is>
       </c>
       <c r="AG633" t="n">
@@ -68854,7 +68854,7 @@
       </c>
       <c r="AF638" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG638" t="n">
@@ -69292,7 +69292,7 @@
       </c>
       <c r="AF642" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG642" t="n">
@@ -69591,7 +69591,7 @@
       </c>
       <c r="AF645" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG645" t="n">
@@ -69695,7 +69695,7 @@
       </c>
       <c r="AF646" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG646" t="n">
@@ -70162,7 +70162,7 @@
       </c>
       <c r="AF650" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG650" t="n">
@@ -70453,7 +70453,7 @@
       </c>
       <c r="AF653" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG653" t="n">
@@ -70562,7 +70562,7 @@
       </c>
       <c r="AF654" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG654" t="n">
@@ -70666,7 +70666,7 @@
       </c>
       <c r="AF655" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG655" t="n">
@@ -71092,7 +71092,7 @@
       </c>
       <c r="AF659" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG659" t="n">
@@ -71196,7 +71196,7 @@
       </c>
       <c r="AF660" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG660" t="n">
@@ -71814,7 +71814,7 @@
       </c>
       <c r="AF666" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG666" t="n">
@@ -72151,7 +72151,7 @@
       </c>
       <c r="AF669" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Velox Express</t>
         </is>
       </c>
       <c r="AG669" t="n">
@@ -72255,7 +72255,7 @@
       </c>
       <c r="AF670" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG670" t="n">
@@ -73544,7 +73544,7 @@
       </c>
       <c r="AF682" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG682" t="n">
@@ -75479,7 +75479,7 @@
       </c>
       <c r="AF699" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG699" t="n">
@@ -75687,7 +75687,7 @@
       </c>
       <c r="AF701" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Velox Express</t>
         </is>
       </c>
       <c r="AG701" t="n">
@@ -76128,7 +76128,7 @@
       </c>
       <c r="AF705" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG705" t="n">
@@ -76559,7 +76559,7 @@
       </c>
       <c r="AF709" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG709" t="n">
@@ -77293,7 +77293,7 @@
       </c>
       <c r="AF716" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG716" t="n">
@@ -77397,7 +77397,7 @@
       </c>
       <c r="AF717" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG717" t="n">
@@ -77600,7 +77600,7 @@
       </c>
       <c r="AF719" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG719" t="n">
@@ -78345,7 +78345,7 @@
       </c>
       <c r="AF726" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG726" t="n">
@@ -78454,7 +78454,7 @@
       </c>
       <c r="AF727" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Velox Express</t>
         </is>
       </c>
       <c r="AG727" t="n">
@@ -78558,7 +78558,7 @@
       </c>
       <c r="AF728" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG728" t="n">
@@ -78758,7 +78758,7 @@
       </c>
       <c r="AF730" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Velox Express</t>
         </is>
       </c>
       <c r="AG730" t="n">
@@ -79938,7 +79938,7 @@
       </c>
       <c r="AF741" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG741" t="n">
@@ -80343,7 +80343,7 @@
       </c>
       <c r="AF745" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG745" t="n">
@@ -80447,7 +80447,7 @@
       </c>
       <c r="AF746" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Velox Express</t>
         </is>
       </c>
       <c r="AG746" t="n">
@@ -80551,7 +80551,7 @@
       </c>
       <c r="AF747" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG747" t="n">
@@ -80987,7 +80987,7 @@
       </c>
       <c r="AF751" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Velox Express</t>
         </is>
       </c>
       <c r="AG751" t="n">
@@ -81091,7 +81091,7 @@
       </c>
       <c r="AF752" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Velox Express</t>
         </is>
       </c>
       <c r="AG752" t="n">
@@ -81628,7 +81628,7 @@
       </c>
       <c r="AF757" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG757" t="n">
@@ -81732,7 +81732,7 @@
       </c>
       <c r="AF758" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG758" t="n">
@@ -81836,7 +81836,7 @@
       </c>
       <c r="AF759" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG759" t="n">
@@ -81940,7 +81940,7 @@
       </c>
       <c r="AF760" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG760" t="n">
@@ -82148,7 +82148,7 @@
       </c>
       <c r="AF762" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG762" t="n">
@@ -83055,7 +83055,7 @@
       </c>
       <c r="AF770" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG770" t="n">
@@ -83159,7 +83159,7 @@
       </c>
       <c r="AF771" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG771" t="n">
@@ -84344,7 +84344,7 @@
       </c>
       <c r="AF782" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Velox Express</t>
         </is>
       </c>
       <c r="AG782" t="n">
@@ -84795,7 +84795,7 @@
       </c>
       <c r="AF786" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG786" t="n">
@@ -85457,7 +85457,7 @@
       </c>
       <c r="AF792" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG792" t="n">
@@ -85569,7 +85569,7 @@
       </c>
       <c r="AF793" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG793" t="n">
@@ -85673,7 +85673,7 @@
       </c>
       <c r="AF794" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG794" t="n">
@@ -86189,7 +86189,7 @@
       </c>
       <c r="AF799" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Velox Express</t>
         </is>
       </c>
       <c r="AG799" t="n">
@@ -86293,7 +86293,7 @@
       </c>
       <c r="AF800" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Velox Express</t>
         </is>
       </c>
       <c r="AG800" t="n">
@@ -86397,7 +86397,7 @@
       </c>
       <c r="AF801" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG801" t="n">
@@ -86605,7 +86605,7 @@
       </c>
       <c r="AF803" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG803" t="n">
@@ -87320,7 +87320,7 @@
       </c>
       <c r="AF809" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG809" t="n">
@@ -87728,7 +87728,7 @@
       </c>
       <c r="AF813" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG813" t="n">
@@ -88174,7 +88174,7 @@
       </c>
       <c r="AF817" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Velox Express</t>
         </is>
       </c>
       <c r="AG817" t="n">
@@ -89095,7 +89095,7 @@
       </c>
       <c r="AF826" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG826" t="n">
@@ -89440,7 +89440,7 @@
       </c>
       <c r="AF829" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG829" t="n">
@@ -90174,7 +90174,7 @@
       </c>
       <c r="AF836" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG836" t="n">
@@ -90387,7 +90387,7 @@
       </c>
       <c r="AF838" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG838" t="n">
@@ -90496,7 +90496,7 @@
       </c>
       <c r="AF839" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG839" t="n">
@@ -91051,7 +91051,7 @@
       </c>
       <c r="AF844" t="inlineStr">
         <is>
-          <t>ColisExpress</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG844" t="n">
@@ -91391,7 +91391,7 @@
       </c>
       <c r="AF847" t="inlineStr">
         <is>
-          <t>TransEuro</t>
+          <t>Velox Express</t>
         </is>
       </c>
       <c r="AG847" t="n">
@@ -91503,7 +91503,7 @@
       </c>
       <c r="AF848" t="inlineStr">
         <is>
-          <t>RapidPost</t>
+          <t>Noria Standard</t>
         </is>
       </c>
       <c r="AG848" t="n">

</xml_diff>